<commit_message>
Drop duplicate Sub-mode Prevention/Detection columns in merge-mode
Prevention now gets the same A/B split treatment as Severity/Detection
in merge-mode, so Sub-mode Prevention and Sub-mode Detection were just
repeating text already shown in Prevention/Detection Note. Remove both
columns when --merge-mode is on; non-merge-mode output is unaffected.
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV29"/>
+  <dimension ref="A1:AT29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1623,9 +1623,7 @@
     <col width="40" customWidth="1" min="43" max="43"/>
     <col width="45" customWidth="1" min="44" max="44"/>
     <col width="35" customWidth="1" min="45" max="45"/>
-    <col width="45" customWidth="1" min="46" max="46"/>
-    <col width="45" customWidth="1" min="47" max="47"/>
-    <col width="50" customWidth="1" min="48" max="48"/>
+    <col width="50" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2068,8 +2066,6 @@
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
       <c r="AT13" s="205" t="n"/>
-      <c r="AU13" s="205" t="n"/>
-      <c r="AV13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2118,8 +2114,6 @@
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
       <c r="AT14" s="205" t="n"/>
-      <c r="AU14" s="205" t="n"/>
-      <c r="AV14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2313,16 +2307,6 @@
         </is>
       </c>
       <c r="AT15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-mode Prevention</t>
-        </is>
-      </c>
-      <c r="AU15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-mode Detection</t>
-        </is>
-      </c>
-      <c r="AV15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -2375,8 +2359,6 @@
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
       <c r="AT16" s="208" t="n"/>
-      <c r="AU16" s="208" t="n"/>
-      <c r="AV16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2425,8 +2407,6 @@
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
       <c r="AT17" s="208" t="n"/>
-      <c r="AU17" s="208" t="n"/>
-      <c r="AV17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2574,7 +2554,8 @@
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: add soft-lined, dedicated headlamp nests and protective lens films/caps on parts and trolleys to prevent contact with hard edges during handling and alignment.</t>
+          <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: apply a removable protective film to the headlamp lens from storage through installation, with a poka‑yoke removal step at final inspection to prevent handling scratches.
+B = The plant's recorded Cause does not match this Mode; addressing the more plausible damage mechanism instead: add a padded alignment/installation fixture with hard locating stops to support the headlamp and prevent lens/housing contact with the BIW during fitment and tightening.</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
@@ -2584,18 +2565,6 @@
         </is>
       </c>
       <c r="AT18" s="223" t="inlineStr">
-        <is>
-          <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: apply a removable protective film to the headlamp lens from storage through installation, with a poka‑yoke removal step at final inspection to prevent handling scratches.
-B = The plant's recorded Cause does not match this Mode; addressing the more plausible damage mechanism instead: add a padded alignment/installation fixture with hard locating stops to support the headlamp and prevent lens/housing contact with the BIW during fitment and tightening.</t>
-        </is>
-      </c>
-      <c r="AU18" s="223" t="inlineStr">
-        <is>
-          <t>A = Add a machine‑vision inspection with controlled lighting to detect lens scratches and interlock the station to automatically reject discrepant headlamps.
-B = Add an in-station automated functional illumination test that powers the headlamp and measures current and lux with go/no-go limits to catch 'does not turn ON' and 'dim' before release.</t>
-        </is>
-      </c>
-      <c r="AV18" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
@@ -2654,8 +2623,6 @@
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
       <c r="AT19" s="223" t="n"/>
-      <c r="AU19" s="223" t="n"/>
-      <c r="AV19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2724,7 +2691,8 @@
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>Add VIN-driven bin lockout on the headlamp sequencing trolley so only the correct headlamp variant bin opens for the current vehicle, preventing wrong-part selection at pickup.</t>
+          <t>A = Add a VIN-driven pick-to-light/scan-interlocked sequencing trolley that only enables the correct headlamp bin for the build and alarms/locks the process if any other bin is accessed to prevent wrong-part picks.
+B = Add a barcode/RFID scan interlock tied to the build manifest that only enables the torque tool and allows installation when the scanned headlamp part number matches the vehicle model at this station.</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
@@ -2734,18 +2702,6 @@
         </is>
       </c>
       <c r="AT20" s="223" t="inlineStr">
-        <is>
-          <t>A = Add a VIN-driven pick-to-light/scan-interlocked sequencing trolley that only enables the correct headlamp bin for the build and alarms/locks the process if any other bin is accessed to prevent wrong-part picks.
-B = Add a barcode/RFID scan interlock tied to the build manifest that only enables the torque tool and allows installation when the scanned headlamp part number matches the vehicle model at this station.</t>
-        </is>
-      </c>
-      <c r="AU20" s="223" t="inlineStr">
-        <is>
-          <t>A = Use an in-station DC torque tool with transducer and PLC OK/NOK lockout to verify 6 Nm on each headlamp fastener and prevent release if torque is not achieved (detecting non-firm fitment).
-B = Implement an automated in-station headlamp functional test that powers the lamp after connection and measures current/illumination with sensors, stopping the line and flagging a mismatch if the unit is off or out of spec.</t>
-        </is>
-      </c>
-      <c r="AV20" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2802,8 +2758,6 @@
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
       <c r="AT21" s="223" t="n"/>
-      <c r="AU21" s="223" t="n"/>
-      <c r="AV21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2884,9 +2838,7 @@
         </is>
       </c>
       <c r="AS22" s="223" t="inlineStr"/>
-      <c r="AT22" s="223" t="inlineStr"/>
-      <c r="AU22" s="223" t="inlineStr"/>
-      <c r="AV22" s="223" t="inlineStr">
+      <c r="AT22" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2963,8 +2915,6 @@
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
       <c r="AT23" s="223" t="n"/>
-      <c r="AU23" s="223" t="n"/>
-      <c r="AV23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -3035,9 +2985,7 @@
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr"/>
-      <c r="AT24" s="223" t="inlineStr"/>
-      <c r="AU24" s="223" t="inlineStr"/>
-      <c r="AV24" s="223" t="inlineStr">
+      <c r="AT24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -3098,8 +3046,6 @@
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
       <c r="AT25" s="223" t="n"/>
-      <c r="AU25" s="223" t="n"/>
-      <c r="AV25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3186,7 +3132,8 @@
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>Add a pin-locating/stop fixture to set the headlamp-to-fender gap and a torque tool with screw-count and 6 Nm OK interlock that prevents job completion if any headlamp screw is missing or out of spec.</t>
+          <t>A = Add a datum-based alignment/locator fixture with hard edge stops and hole locators to set the headlamp-to-fender gap and align the screw bosses before fastening so screws can be fitted correctly every time.
+B = Add a dedicated locating/positioning fixture or hard datum pins at the headlamp mounting points to set flushness and gap to spec before torquing, preventing misalignment by design.</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
@@ -3196,18 +3143,6 @@
         </is>
       </c>
       <c r="AT26" s="223" t="inlineStr">
-        <is>
-          <t>A = Add a datum-based alignment/locator fixture with hard edge stops and hole locators to set the headlamp-to-fender gap and align the screw bosses before fastening so screws can be fitted correctly every time.
-B = Add a dedicated locating/positioning fixture or hard datum pins at the headlamp mounting points to set flushness and gap to spec before torquing, preventing misalignment by design.</t>
-        </is>
-      </c>
-      <c r="AU26" s="223" t="inlineStr">
-        <is>
-          <t>A = Use an electronic torque controller that counts each fastener and verifies torque/angle OK for all required screws, blocking proceed on any missing/under/over-torqued condition.
-B = Install an in-station camera-based gap/flushness measurement system interlocked to the station (block OK-to-release if any measured gap/flushness is out of spec).</t>
-        </is>
-      </c>
-      <c r="AV26" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
         </is>
@@ -3274,8 +3209,6 @@
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
       <c r="AT27" s="223" t="n"/>
-      <c r="AU27" s="223" t="n"/>
-      <c r="AV27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3359,9 +3292,7 @@
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr"/>
-      <c r="AT28" s="223" t="inlineStr"/>
-      <c r="AU28" s="223" t="inlineStr"/>
-      <c r="AV28" s="223" t="inlineStr">
+      <c r="AT28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3432,7 +3363,8 @@
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>Replace the current setup with a DC electric torque tool locked at 6 Nm with torque/angle control and socket/tool-ID poka‑yoke to prevent wrong tool use and eliminate operator-set errors.</t>
+          <t>A = Install a DC electric nutrunner with controller‑locked 6 Nm program and RFID/tool‑ID lockout so the station cannot run with the wrong tool or setting, directly addressing operator mistake and wrong/miscalibrated tool causes.
+B = Install a DC torque-controlled driver locked to a 6 Nm window with OK/NOK lockout (paired to this station/tool ID) to prevent over‑torque from operator error, wrong tool use, or drift.</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
@@ -3443,25 +3375,13 @@
       </c>
       <c r="AT29" s="223" t="inlineStr">
         <is>
-          <t>A = Install a DC electric nutrunner with controller‑locked 6 Nm program and RFID/tool‑ID lockout so the station cannot run with the wrong tool or setting, directly addressing operator mistake and wrong/miscalibrated tool causes.
-B = Install a DC torque-controlled driver locked to a 6 Nm window with OK/NOK lockout (paired to this station/tool ID) to prevent over‑torque from operator error, wrong tool use, or drift.</t>
-        </is>
-      </c>
-      <c r="AU29" s="223" t="inlineStr">
-        <is>
-          <t>A = Integrate in‑station torque monitoring (nutrunner torque‑angle OK/NOK with PLC interlock) so the station cannot advance unless each fastener achieves the 6 Nm OK result.
-B = Integrate in‑station electronic torque monitoring with data logging and an interlock that blocks job release if the recorded torque is outside the 6 Nm window (OK/NOK confirmation).</t>
-        </is>
-      </c>
-      <c r="AV29" s="223" t="inlineStr">
-        <is>
           <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="181">
+  <mergeCells count="169">
     <mergeCell ref="AP18:AP19"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
@@ -3470,7 +3390,6 @@
     <mergeCell ref="AM15:AM17"/>
     <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
-    <mergeCell ref="AV18:AV19"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
@@ -3481,20 +3400,18 @@
     <mergeCell ref="T13:AA14"/>
     <mergeCell ref="S1:T2"/>
     <mergeCell ref="D12:F12"/>
-    <mergeCell ref="AU24:AU25"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G13:L14"/>
     <mergeCell ref="AR24:AR25"/>
     <mergeCell ref="K9:T9"/>
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
-    <mergeCell ref="AU26:AU27"/>
     <mergeCell ref="AN15:AN17"/>
     <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
-    <mergeCell ref="AU18:AU19"/>
+    <mergeCell ref="AM13:AT14"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3514,9 +3431,7 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
-    <mergeCell ref="AM13:AV14"/>
     <mergeCell ref="AT15:AT17"/>
-    <mergeCell ref="AV15:AV17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
@@ -3552,7 +3467,6 @@
     <mergeCell ref="AC15:AC17"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
-    <mergeCell ref="AV20:AV21"/>
     <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AS24:AS25"/>
     <mergeCell ref="AD15:AD17"/>
@@ -3564,9 +3478,7 @@
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
     <mergeCell ref="AS20:AS21"/>
-    <mergeCell ref="AU20:AU21"/>
     <mergeCell ref="AP24:AP25"/>
-    <mergeCell ref="AV22:AV23"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
@@ -3588,15 +3500,12 @@
     <mergeCell ref="AM20:AM21"/>
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
-    <mergeCell ref="AV24:AV25"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
     <mergeCell ref="AT22:AT23"/>
-    <mergeCell ref="AV26:AV27"/>
     <mergeCell ref="T19:U19"/>
-    <mergeCell ref="AU15:AU17"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
@@ -3639,7 +3548,6 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="AU22:AU23"/>
     <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>

</xml_diff>

<commit_message>
Drop Sub-modes column in merge-mode; it duplicated the Failure Mode cell
The plant's own Failure Mode column already shows the raw merged text
with both sub-modes in it, so merge-mode's separate "Sub-modes" column
("A = <name> / B = <name>") was just restating that. The A/B labels now
only appear where the actual per-mode values live: Severity, Detection,
and Prevention. Also fixes the Remark note that referenced the now-gone
Sub-modes column. Non-merge-mode output is unaffected (verified byte-
identical to before).
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT29"/>
+  <dimension ref="A1:AS29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1622,8 +1622,7 @@
     <col width="8" customWidth="1" min="42" max="42"/>
     <col width="40" customWidth="1" min="43" max="43"/>
     <col width="45" customWidth="1" min="44" max="44"/>
-    <col width="35" customWidth="1" min="45" max="45"/>
-    <col width="50" customWidth="1" min="46" max="46"/>
+    <col width="50" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2065,7 +2064,6 @@
       <c r="AQ13" s="205" t="n"/>
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
-      <c r="AT13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2113,7 +2111,6 @@
       <c r="AQ14" s="205" t="n"/>
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
-      <c r="AT14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2302,11 +2299,6 @@
         </is>
       </c>
       <c r="AS15" s="208" t="inlineStr">
-        <is>
-          <t>Sub-modes</t>
-        </is>
-      </c>
-      <c r="AT15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -2358,7 +2350,6 @@
       <c r="AQ16" s="208" t="n"/>
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
-      <c r="AT16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2406,7 +2397,6 @@
       <c r="AQ17" s="208" t="n"/>
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
-      <c r="AT17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2560,13 +2550,7 @@
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>A = Scratch on headlamp
-B = Damage on headlamp</t>
-        </is>
-      </c>
-      <c r="AT18" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2622,7 +2606,6 @@
       <c r="AQ19" s="223" t="n"/>
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
-      <c r="AT19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2697,13 +2680,7 @@
       </c>
       <c r="AS20" s="223" t="inlineStr">
         <is>
-          <t>A = Fitment is not firm
-B = Wrong selection of headlamp (not as per model)</t>
-        </is>
-      </c>
-      <c r="AT20" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2734,6 @@
       <c r="AQ21" s="223" t="n"/>
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
-      <c r="AT21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2837,8 +2813,7 @@
           <t>Add a connector-lock poka‑yoke: a mechanical go/no‑go gauge or latch‑position sensor interlocked with the station PLC so the cycle cannot complete unless the connector latch is fully engaged.</t>
         </is>
       </c>
-      <c r="AS22" s="223" t="inlineStr"/>
-      <c r="AT22" s="223" t="inlineStr">
+      <c r="AS22" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2914,7 +2889,6 @@
       <c r="AQ23" s="223" t="n"/>
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
-      <c r="AT23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -2984,8 +2958,7 @@
           <t>Add a DC electric nutrunner with torque/angle monitoring and an OK-to-proceed interlock that requires both headlamp bolts to be run to 6 Nm (correct count and torque achieved) before allowing the station to complete.</t>
         </is>
       </c>
-      <c r="AS24" s="223" t="inlineStr"/>
-      <c r="AT24" s="223" t="inlineStr">
+      <c r="AS24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -3045,7 +3018,6 @@
       <c r="AQ25" s="223" t="n"/>
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
-      <c r="AT25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3138,13 +3110,7 @@
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>A = Failed to fit screws
-B = Not maintained gap</t>
-        </is>
-      </c>
-      <c r="AT26" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
+          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3174,6 @@
       <c r="AQ27" s="223" t="n"/>
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
-      <c r="AT27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3291,8 +3256,7 @@
           <t>Add a station interlock with tool-ID/torque-program lock (RFID/barcode pairing) so only the correct, calibrated 6 Nm power tool can run this joint and its torque setting cannot be changed by the operator.</t>
         </is>
       </c>
-      <c r="AS28" s="223" t="inlineStr"/>
-      <c r="AT28" s="223" t="inlineStr">
+      <c r="AS28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3369,32 +3333,23 @@
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>A = Torque not achieved
-B = Over torque</t>
-        </is>
-      </c>
-      <c r="AT29" s="223" t="inlineStr">
-        <is>
-          <t>Merged failure mode (2 distinct modes detected) - see Sub-modes columns for per-mode Severity/Detection/actions. Row-level Severity/Detection above are the worst case; consider splitting this row in the plant sheet. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="163">
     <mergeCell ref="AP18:AP19"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
-    <mergeCell ref="AT24:AT25"/>
     <mergeCell ref="AM15:AM17"/>
-    <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
     <mergeCell ref="O23:O25"/>
-    <mergeCell ref="AT20:AT21"/>
     <mergeCell ref="M26:N29"/>
     <mergeCell ref="W15:X17"/>
     <mergeCell ref="T13:AA14"/>
@@ -3407,11 +3362,9 @@
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
     <mergeCell ref="AN15:AN17"/>
-    <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
-    <mergeCell ref="AM13:AT14"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3431,7 +3384,6 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
-    <mergeCell ref="AT15:AT17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
@@ -3483,6 +3435,7 @@
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
     <mergeCell ref="G11:H11"/>
+    <mergeCell ref="AM13:AS14"/>
     <mergeCell ref="AH15:AH17"/>
     <mergeCell ref="AS22:AS23"/>
     <mergeCell ref="AJ15:AJ17"/>
@@ -3504,7 +3457,6 @@
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
-    <mergeCell ref="AT22:AT23"/>
     <mergeCell ref="T19:U19"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>

</xml_diff>

<commit_message>
Add Failure Mode as the first Suggestion-block column, both formats
The sheet's own Failure Mode column sits far to the left of the
Suggestion block, so a reader scrolled over to Severity/Detection/
Prevention had no easy way to tell which mode(s) those values were even
about - especially once split into "A = .../B = ...". Repeat the mode
name(s) right at the start of the block instead: plain text for a single
mode, "A = <name>\nB = <name>" for a merged/split one. Applies to both
--merge-mode and the plain output, so both committed suggestion Excels
are regenerated (their other columns are unaffected).
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -1611,18 +1611,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS29"/>
+  <dimension ref="A1:AT29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
     <col width="12.5703125" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="39" max="39"/>
-    <col width="45" customWidth="1" min="40" max="40"/>
-    <col width="8" customWidth="1" min="41" max="41"/>
+    <col width="35" customWidth="1" min="39" max="39"/>
+    <col width="8" customWidth="1" min="40" max="40"/>
+    <col width="45" customWidth="1" min="41" max="41"/>
     <col width="8" customWidth="1" min="42" max="42"/>
-    <col width="40" customWidth="1" min="43" max="43"/>
-    <col width="45" customWidth="1" min="44" max="44"/>
-    <col width="50" customWidth="1" min="45" max="45"/>
+    <col width="8" customWidth="1" min="43" max="43"/>
+    <col width="40" customWidth="1" min="44" max="44"/>
+    <col width="45" customWidth="1" min="45" max="45"/>
+    <col width="50" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2064,6 +2065,7 @@
       <c r="AQ13" s="205" t="n"/>
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
+      <c r="AT13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2111,6 +2113,7 @@
       <c r="AQ14" s="205" t="n"/>
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
+      <c r="AT14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2270,35 +2273,40 @@
       </c>
       <c r="AM15" s="208" t="inlineStr">
         <is>
+          <t>Failure Mode</t>
+        </is>
+      </c>
+      <c r="AN15" s="208" t="inlineStr">
+        <is>
           <t>Severity (S)</t>
         </is>
       </c>
-      <c r="AN15" s="208" t="inlineStr">
+      <c r="AO15" s="208" t="inlineStr">
         <is>
           <t>Severity Note</t>
         </is>
       </c>
-      <c r="AO15" s="208" t="inlineStr">
+      <c r="AP15" s="208" t="inlineStr">
         <is>
           <t>Occurrence (O)</t>
         </is>
       </c>
-      <c r="AP15" s="208" t="inlineStr">
+      <c r="AQ15" s="208" t="inlineStr">
         <is>
           <t>Detection (D)</t>
         </is>
       </c>
-      <c r="AQ15" s="208" t="inlineStr">
+      <c r="AR15" s="208" t="inlineStr">
         <is>
           <t>Detection Note</t>
         </is>
       </c>
-      <c r="AR15" s="208" t="inlineStr">
+      <c r="AS15" s="208" t="inlineStr">
         <is>
           <t>Prevention</t>
         </is>
       </c>
-      <c r="AS15" s="208" t="inlineStr">
+      <c r="AT15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
@@ -2350,6 +2358,7 @@
       <c r="AQ16" s="208" t="n"/>
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
+      <c r="AT16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2397,6 +2406,7 @@
       <c r="AQ17" s="208" t="n"/>
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
+      <c r="AT17" s="208" t="n"/>
     </row>
     <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2520,35 +2530,41 @@
       <c r="AL18" s="35" t="n"/>
       <c r="AM18" s="223" t="inlineStr">
         <is>
+          <t>A = Scratch on headlamp
+B = Damage on headlamp</t>
+        </is>
+      </c>
+      <c r="AN18" s="223" t="inlineStr">
+        <is>
           <t>A = 7
 B = 8</t>
         </is>
       </c>
-      <c r="AN18" s="223" t="inlineStr">
+      <c r="AO18" s="223" t="inlineStr">
         <is>
           <t>A = The applicable End User effect "Insufficient brightness / dim light" describes degraded primary lighting performance due to a scratched lens, which matches the table’s definition for Severity 7 (degradation of a primary vehicle function).
 B = End User effects list 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation); no safety or regulatory wording is provided. Because the mode is 'Damage on headlamp' and can directly cause either, the worst-case direct outcome is loss of the primary lighting function (S=8).</t>
         </is>
       </c>
-      <c r="AP18" s="223" t="inlineStr">
+      <c r="AQ18" s="223" t="inlineStr">
         <is>
           <t>A = 8
 B = 8</t>
         </is>
       </c>
-      <c r="AQ18" s="223" t="inlineStr">
+      <c r="AR18" s="223" t="inlineStr">
         <is>
           <t>A = Add a machine‑vision inspection with controlled lighting to detect lens scratches and interlock the station to automatically reject discrepant headlamps.
 B = Add an in-station automated functional illumination test that powers the headlamp and measures current and lux with go/no-go limits to catch 'does not turn ON' and 'dim' before release.</t>
         </is>
       </c>
-      <c r="AR18" s="223" t="inlineStr">
+      <c r="AS18" s="223" t="inlineStr">
         <is>
           <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: apply a removable protective film to the headlamp lens from storage through installation, with a poka‑yoke removal step at final inspection to prevent handling scratches.
 B = The plant's recorded Cause does not match this Mode; addressing the more plausible damage mechanism instead: add a padded alignment/installation fixture with hard locating stops to support the headlamp and prevent lens/housing contact with the BIW during fitment and tightening.</t>
         </is>
       </c>
-      <c r="AS18" s="223" t="inlineStr">
+      <c r="AT18" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
@@ -2602,10 +2618,11 @@
       <c r="AL19" s="35" t="n"/>
       <c r="AM19" s="223" t="n"/>
       <c r="AN19" s="223" t="n"/>
-      <c r="AP19" s="223" t="n"/>
+      <c r="AO19" s="223" t="n"/>
       <c r="AQ19" s="223" t="n"/>
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
+      <c r="AT19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2650,35 +2667,41 @@
       <c r="AL20" s="35" t="n"/>
       <c r="AM20" s="223" t="inlineStr">
         <is>
+          <t>A = Fitment is not firm
+B = Wrong selection of headlamp (not as per model)</t>
+        </is>
+      </c>
+      <c r="AN20" s="223" t="inlineStr">
+        <is>
           <t>A = 8
 B = 8</t>
         </is>
       </c>
-      <c r="AN20" s="223" t="inlineStr">
+      <c r="AO20" s="223" t="inlineStr">
         <is>
           <t>A = The End User effects explicitly state loss or degradation of the headlamp’s primary function (no illumination or dim light). This maps to loss of primary vehicle function (S=8) or degradation of primary function (S=7). Given both are equally plausible for a wrong-part selection, the worst applicable severity is 8.
 B = The listed End User effects for a wrong headlamp selection include both non-operation and dim output, which correspond to total loss or degradation of the headlamp’s primary function; there is no explicit safety or regulatory language, so severity is set by primary-function loss (worst-case S=8).</t>
         </is>
       </c>
-      <c r="AP20" s="223" t="inlineStr">
+      <c r="AQ20" s="223" t="inlineStr">
         <is>
           <t>A = 8
 B = 8</t>
         </is>
       </c>
-      <c r="AQ20" s="223" t="inlineStr">
+      <c r="AR20" s="223" t="inlineStr">
         <is>
           <t>A = Use an in-station DC torque tool with transducer and PLC OK/NOK lockout to verify 6 Nm on each headlamp fastener and prevent release if torque is not achieved (detecting non-firm fitment).
 B = Implement an automated in-station headlamp functional test that powers the lamp after connection and measures current/illumination with sensors, stopping the line and flagging a mismatch if the unit is off or out of spec.</t>
         </is>
       </c>
-      <c r="AR20" s="223" t="inlineStr">
+      <c r="AS20" s="223" t="inlineStr">
         <is>
           <t>A = Add a VIN-driven pick-to-light/scan-interlocked sequencing trolley that only enables the correct headlamp bin for the build and alarms/locks the process if any other bin is accessed to prevent wrong-part picks.
 B = Add a barcode/RFID scan interlock tied to the build manifest that only enables the torque tool and allows installation when the scanned headlamp part number matches the vehicle model at this station.</t>
         </is>
       </c>
-      <c r="AS20" s="223" t="inlineStr">
+      <c r="AT20" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -2730,10 +2753,11 @@
       <c r="AL21" s="35" t="n"/>
       <c r="AM21" s="223" t="n"/>
       <c r="AN21" s="223" t="n"/>
-      <c r="AP21" s="223" t="n"/>
+      <c r="AO21" s="223" t="n"/>
       <c r="AQ21" s="223" t="n"/>
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
+      <c r="AT21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2792,28 +2816,34 @@
       <c r="AJ22" s="45" t="n"/>
       <c r="AK22" s="45" t="n"/>
       <c r="AL22" s="35" t="n"/>
-      <c r="AM22" s="223" t="n">
+      <c r="AM22" s="223" t="inlineStr">
+        <is>
+          <t>IMPROPER LOCKING /
+POOR LOCKING</t>
+        </is>
+      </c>
+      <c r="AN22" s="223" t="n">
         <v>10</v>
       </c>
-      <c r="AN22" s="223" t="inlineStr">
+      <c r="AO22" s="223" t="inlineStr">
         <is>
           <t>The End User effects explicitly list 'Increased risk of accident', which is causally plausible for an unconnected/poorly locked headlamp connector causing the lamp not to turn on and reducing visibility. Per the table, this is a safety/health risk to road users, so Severity is 10.</t>
         </is>
       </c>
-      <c r="AP22" s="223" t="n">
+      <c r="AQ22" s="223" t="n">
         <v>8</v>
       </c>
-      <c r="AQ22" s="223" t="inlineStr">
+      <c r="AR22" s="223" t="inlineStr">
         <is>
           <t>Add an in‑station automated functional test that powers each headlamp and verifies illumination/current draw with a light or current sensor, stopping the process if either lamp fails.</t>
         </is>
       </c>
-      <c r="AR22" s="223" t="inlineStr">
+      <c r="AS22" s="223" t="inlineStr">
         <is>
           <t>Add a connector-lock poka‑yoke: a mechanical go/no‑go gauge or latch‑position sensor interlocked with the station PLC so the cycle cannot complete unless the connector latch is fully engaged.</t>
         </is>
       </c>
-      <c r="AS22" s="223" t="inlineStr">
+      <c r="AT22" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -2885,10 +2915,11 @@
       <c r="AL23" s="10" t="n"/>
       <c r="AM23" s="223" t="n"/>
       <c r="AN23" s="223" t="n"/>
-      <c r="AP23" s="223" t="n"/>
+      <c r="AO23" s="223" t="n"/>
       <c r="AQ23" s="223" t="n"/>
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
+      <c r="AT23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -2937,28 +2968,33 @@
       <c r="AJ24" s="12" t="n"/>
       <c r="AK24" s="12" t="n"/>
       <c r="AL24" s="10" t="n"/>
-      <c r="AM24" s="223" t="n">
+      <c r="AM24" s="223" t="inlineStr">
+        <is>
+          <t>OPERATOR FAILED TO PREFIT BOLTS</t>
+        </is>
+      </c>
+      <c r="AN24" s="223" t="n">
         <v>10</v>
       </c>
-      <c r="AN24" s="223" t="inlineStr">
+      <c r="AO24" s="223" t="inlineStr">
         <is>
           <t>The End User effects explicitly state 'Increased risk of accident,' which is a plausible consequence of an unbolted/misaligned headlamp causing reduced road illumination. Per the scoring rules and Table C2-1, this constitutes an effect that affects safe operation of the vehicle, warranting Severity 10.</t>
         </is>
       </c>
-      <c r="AP24" s="223" t="n">
+      <c r="AQ24" s="223" t="n">
         <v>8</v>
       </c>
-      <c r="AQ24" s="223" t="inlineStr">
+      <c r="AR24" s="223" t="inlineStr">
         <is>
           <t>Install a machine-vision presence/position check at station exit to verify both headlamp bolt heads are present and seated, with automatic NOK stop/reject if either bolt is missing.</t>
         </is>
       </c>
-      <c r="AR24" s="223" t="inlineStr">
+      <c r="AS24" s="223" t="inlineStr">
         <is>
           <t>Add a DC electric nutrunner with torque/angle monitoring and an OK-to-proceed interlock that requires both headlamp bolts to be run to 6 Nm (correct count and torque achieved) before allowing the station to complete.</t>
         </is>
       </c>
-      <c r="AS24" s="223" t="inlineStr">
+      <c r="AT24" s="223" t="inlineStr">
         <is>
           <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
@@ -3014,10 +3050,11 @@
       <c r="AL25" s="10" t="n"/>
       <c r="AM25" s="223" t="n"/>
       <c r="AN25" s="223" t="n"/>
-      <c r="AP25" s="223" t="n"/>
+      <c r="AO25" s="223" t="n"/>
       <c r="AQ25" s="223" t="n"/>
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
+      <c r="AT25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3080,35 +3117,41 @@
       <c r="AL26" s="10" t="n"/>
       <c r="AM26" s="223" t="inlineStr">
         <is>
+          <t>A = Failed to fit screws
+B = Not maintained gap</t>
+        </is>
+      </c>
+      <c r="AN26" s="223" t="inlineStr">
+        <is>
           <t>A = 4
 B = 4</t>
         </is>
       </c>
-      <c r="AN26" s="223" t="inlineStr">
+      <c r="AO26" s="223" t="inlineStr">
         <is>
           <t>A = The direct customer-facing consequence of failing to fit the mounting screws is a loose lamp causing rattling/vibration noise during driving, which aligns with a very objectionable NVH condition per the table.
 B = Among the listed End User effects, water ingress is the direct consequence of an uneven headlamp-to-fender gap and is best characterized as a very objectionable visible condition to the customer; no explicit safety, regulatory, or stated primary-function loss is given.</t>
         </is>
       </c>
-      <c r="AP26" s="223" t="inlineStr">
+      <c r="AQ26" s="223" t="inlineStr">
         <is>
           <t>A = 8
 B = 8</t>
         </is>
       </c>
-      <c r="AQ26" s="223" t="inlineStr">
+      <c r="AR26" s="223" t="inlineStr">
         <is>
           <t>A = Use an electronic torque controller that counts each fastener and verifies torque/angle OK for all required screws, blocking proceed on any missing/under/over-torqued condition.
 B = Install an in-station camera-based gap/flushness measurement system interlocked to the station (block OK-to-release if any measured gap/flushness is out of spec).</t>
         </is>
       </c>
-      <c r="AR26" s="223" t="inlineStr">
+      <c r="AS26" s="223" t="inlineStr">
         <is>
           <t>A = Add a datum-based alignment/locator fixture with hard edge stops and hole locators to set the headlamp-to-fender gap and align the screw bosses before fastening so screws can be fitted correctly every time.
 B = Add a dedicated locating/positioning fixture or hard datum pins at the headlamp mounting points to set flushness and gap to spec before torquing, preventing misalignment by design.</t>
         </is>
       </c>
-      <c r="AS26" s="223" t="inlineStr">
+      <c r="AT26" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
         </is>
@@ -3170,10 +3213,11 @@
       <c r="AL27" s="10" t="n"/>
       <c r="AM27" s="223" t="n"/>
       <c r="AN27" s="223" t="n"/>
-      <c r="AP27" s="223" t="n"/>
+      <c r="AO27" s="223" t="n"/>
       <c r="AQ27" s="223" t="n"/>
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
+      <c r="AT27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3235,28 +3279,33 @@
       <c r="AJ28" s="12" t="n"/>
       <c r="AK28" s="12" t="n"/>
       <c r="AL28" s="10" t="n"/>
-      <c r="AM28" s="223" t="n">
+      <c r="AM28" s="223" t="inlineStr">
+        <is>
+          <t>TORQUE NOT ACHIEVED-UNDER TORQUE</t>
+        </is>
+      </c>
+      <c r="AN28" s="223" t="n">
         <v>4</v>
       </c>
-      <c r="AN28" s="223" t="inlineStr">
+      <c r="AO28" s="223" t="inlineStr">
         <is>
           <t>The only direct customer effect of an under-torqued headlamp mounting is rattling/vibration noise while driving, which is an NVH issue. The list contains no explicit safety or regulatory consequence tied to this mode, so severity aligns with "very objectionable" NVH at S=4.</t>
         </is>
       </c>
-      <c r="AP28" s="223" t="n">
+      <c r="AQ28" s="223" t="n">
         <v>9</v>
       </c>
-      <c r="AQ28" s="223" t="inlineStr">
+      <c r="AR28" s="223" t="inlineStr">
         <is>
           <t>Install a transducerized DC nutrunner or in-line torque/angle monitor that records actual achieved torque and provides OK/NOK with line stop if 6 Nm is not reached.</t>
         </is>
       </c>
-      <c r="AR28" s="223" t="inlineStr">
+      <c r="AS28" s="223" t="inlineStr">
         <is>
           <t>Add a station interlock with tool-ID/torque-program lock (RFID/barcode pairing) so only the correct, calibrated 6 Nm power tool can run this joint and its torque setting cannot be changed by the operator.</t>
         </is>
       </c>
-      <c r="AS28" s="223" t="inlineStr">
+      <c r="AT28" s="223" t="inlineStr">
         <is>
           <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3303,35 +3352,41 @@
       <c r="AL29" s="10" t="n"/>
       <c r="AM29" s="223" t="inlineStr">
         <is>
+          <t>A = Torque not achieved
+B = Over torque</t>
+        </is>
+      </c>
+      <c r="AN29" s="223" t="inlineStr">
+        <is>
           <t>A = 4
 B = 4</t>
         </is>
       </c>
-      <c r="AN29" s="223" t="inlineStr">
+      <c r="AO29" s="223" t="inlineStr">
         <is>
           <t>A = For this torque error, the direct user-facing outcomes are either a cracked/broken lens (over‑torque) or rattling/vibration noise (under‑torque), both of which fit the table’s “very objectionable appearance/sound/vibration/harshness/haptics” definition; no safety, regulatory, or explicit primary-function loss is stated.
 B = The DIRECT End User effect of over‑torque here is a cracked/broken lens, which is best characterized as a very objectionable appearance defect; the other listed effects (burnout, water ingress, rattling, discomfort) require additional unstated steps and are therefore INDIRECT.</t>
         </is>
       </c>
-      <c r="AP29" s="223" t="inlineStr">
+      <c r="AQ29" s="223" t="inlineStr">
         <is>
           <t>A = 9
 B = 9</t>
         </is>
       </c>
-      <c r="AQ29" s="223" t="inlineStr">
+      <c r="AR29" s="223" t="inlineStr">
         <is>
           <t>A = Integrate in‑station torque monitoring (nutrunner torque‑angle OK/NOK with PLC interlock) so the station cannot advance unless each fastener achieves the 6 Nm OK result.
 B = Integrate in‑station electronic torque monitoring with data logging and an interlock that blocks job release if the recorded torque is outside the 6 Nm window (OK/NOK confirmation).</t>
         </is>
       </c>
-      <c r="AR29" s="223" t="inlineStr">
+      <c r="AS29" s="223" t="inlineStr">
         <is>
           <t>A = Install a DC electric nutrunner with controller‑locked 6 Nm program and RFID/tool‑ID lockout so the station cannot run with the wrong tool or setting, directly addressing operator mistake and wrong/miscalibrated tool causes.
 B = Install a DC torque-controlled driver locked to a 6 Nm window with OK/NOK lockout (paired to this station/tool ID) to prevent over‑torque from operator error, wrong tool use, or drift.</t>
         </is>
       </c>
-      <c r="AS29" s="223" t="inlineStr">
+      <c r="AT29" s="223" t="inlineStr">
         <is>
           <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
@@ -3339,17 +3394,19 @@
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="163">
-    <mergeCell ref="AP18:AP19"/>
+  <mergeCells count="169">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
+    <mergeCell ref="AT24:AT25"/>
     <mergeCell ref="AM15:AM17"/>
+    <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
     <mergeCell ref="O23:O25"/>
+    <mergeCell ref="AT20:AT21"/>
     <mergeCell ref="M26:N29"/>
     <mergeCell ref="W15:X17"/>
     <mergeCell ref="T13:AA14"/>
@@ -3362,9 +3419,11 @@
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
     <mergeCell ref="AN15:AN17"/>
+    <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
+    <mergeCell ref="AM13:AT14"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3384,11 +3443,11 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
+    <mergeCell ref="AT15:AT17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="AN20:AN21"/>
-    <mergeCell ref="AP20:AP21"/>
     <mergeCell ref="AQ22:AQ23"/>
     <mergeCell ref="AN26:AN27"/>
     <mergeCell ref="A5:C5"/>
@@ -3397,7 +3456,6 @@
     <mergeCell ref="Z18:Z21"/>
     <mergeCell ref="T25:U25"/>
     <mergeCell ref="AN22:AN23"/>
-    <mergeCell ref="AP22:AP23"/>
     <mergeCell ref="P18:Q19"/>
     <mergeCell ref="AQ15:AQ17"/>
     <mergeCell ref="Y23:Y25"/>
@@ -3430,20 +3488,18 @@
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
     <mergeCell ref="AS20:AS21"/>
-    <mergeCell ref="AP24:AP25"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
     <mergeCell ref="G11:H11"/>
-    <mergeCell ref="AM13:AS14"/>
     <mergeCell ref="AH15:AH17"/>
     <mergeCell ref="AS22:AS23"/>
     <mergeCell ref="AJ15:AJ17"/>
     <mergeCell ref="O27:O29"/>
-    <mergeCell ref="AP26:AP27"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="O18:O21"/>
     <mergeCell ref="M18:N21"/>
+    <mergeCell ref="AO18:AO19"/>
     <mergeCell ref="AN18:AN19"/>
     <mergeCell ref="A1:R2"/>
     <mergeCell ref="AL15:AL17"/>
@@ -3454,9 +3510,11 @@
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
     <mergeCell ref="R22:S22"/>
+    <mergeCell ref="AO22:AO23"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
+    <mergeCell ref="AT22:AT23"/>
     <mergeCell ref="T19:U19"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
@@ -3483,10 +3541,12 @@
     <mergeCell ref="AM24:AM25"/>
     <mergeCell ref="M13:S14"/>
     <mergeCell ref="P24:Q25"/>
+    <mergeCell ref="AO24:AO25"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="Z15:Z17"/>
     <mergeCell ref="AQ18:AQ19"/>
     <mergeCell ref="AB15:AB17"/>
+    <mergeCell ref="AO20:AO21"/>
     <mergeCell ref="R21:S21"/>
     <mergeCell ref="T21:U21"/>
     <mergeCell ref="A10:C10"/>
@@ -3496,6 +3556,7 @@
     <mergeCell ref="Y15:Y17"/>
     <mergeCell ref="P26:Q27"/>
     <mergeCell ref="T26:U26"/>
+    <mergeCell ref="AO26:AO27"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>

</xml_diff>

<commit_message>
Build final merge-mode Excel with projected Detection score and row completeness notes
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT29"/>
+  <dimension ref="A1:AV29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1624,6 +1624,8 @@
     <col width="40" customWidth="1" min="44" max="44"/>
     <col width="45" customWidth="1" min="45" max="45"/>
     <col width="50" customWidth="1" min="46" max="46"/>
+    <col width="45" customWidth="1" min="47" max="47"/>
+    <col width="35" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2066,6 +2068,8 @@
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
       <c r="AT13" s="205" t="n"/>
+      <c r="AU13" s="205" t="n"/>
+      <c r="AV13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2114,13 +2118,37 @@
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
       <c r="AT14" s="205" t="n"/>
+      <c r="AU14" s="205" t="n"/>
+      <c r="AV14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -2139,8 +2167,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -2309,6 +2359,16 @@
       <c r="AT15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+      <c r="AU15" s="208" t="inlineStr">
+        <is>
+          <t>AI Review</t>
+        </is>
+      </c>
+      <c r="AV15" s="208" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
         </is>
       </c>
     </row>
@@ -2359,6 +2419,8 @@
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
       <c r="AT16" s="208" t="n"/>
+      <c r="AU16" s="208" t="n"/>
+      <c r="AV16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2407,8 +2469,10 @@
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
       <c r="AT17" s="208" t="n"/>
-    </row>
-    <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
+      <c r="AU17" s="208" t="n"/>
+      <c r="AV17" s="208" t="n"/>
+    </row>
+    <row r="18" ht="142.5" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
         <is>
           <t>HEAD LAMP STAGE</t>
@@ -2417,36 +2481,293 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 RH / LH HEAD LAMP FITMENT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Connections, Bolt fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 Headlamp assembly in specific design (bulb/LED assembly, lens fitting, aiming, electrical connection)
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Provide adequate illumination of the road ahead during low-light or night conditions
 2. Ensure visibility of the vehicle to other road users
 3. Meet legal/regulatory lighting requirements (beam pattern, intensity, color)</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -2458,32 +2779,185 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. COLLECT THE HEAD LAMP LH / RH SIDE FROM STORAGE AREA AND SCAN THE PART
 2. CONNECT THE 2 CONNECTORS WITH HEAD LAMP
 3. ALIGN THE HEAD LAMP WITH THE BIW AND THEN TIGHT WITH BOLTS
-2. Machine:
-Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Head lamp from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Head lamp from sequencing trolley and scan
 2. Align H/L with BIW, then do the connections with wiring harness with head lamp and tight with bolts
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong Head lamp variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Lens cracked or broken
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Headlamp does not turn ON
 2. Insufficient brightness / dim light
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -2530,8 +3004,8 @@
       <c r="AL18" s="35" t="n"/>
       <c r="AM18" s="223" t="inlineStr">
         <is>
-          <t>A = Scratch on headlamp
-B = Damage on headlamp</t>
+          <t>A = SCRATCH
+B = DAMAGE</t>
         </is>
       </c>
       <c r="AN18" s="223" t="inlineStr">
@@ -2542,8 +3016,8 @@
       </c>
       <c r="AO18" s="223" t="inlineStr">
         <is>
-          <t>A = The applicable End User effect "Insufficient brightness / dim light" describes degraded primary lighting performance due to a scratched lens, which matches the table’s definition for Severity 7 (degradation of a primary vehicle function).
-B = End User effects list 'Headlamp does not turn ON' (total loss) and 'Insufficient brightness / dim light' (degradation); no safety or regulatory wording is provided. Because the mode is 'Damage on headlamp' and can directly cause either, the worst-case direct outcome is loss of the primary lighting function (S=8).</t>
+          <t>A = Among the listed End User effects, a scratched headlamp lens most directly leads to "Insufficient brightness / dim light", which is a degradation of the primary lighting function. No explicit safety or regulatory language is stated, and "does not turn on" would require an additional electrical fault not described for a scratch.
+B = The End User effects include "Headlamp does not turn ON" (total loss of the headlamp’s primary function) and "Insufficient brightness / dim light" (degradation). With the Mode "DAMAGE" unspecified, both are plausible direct outcomes; per the worst-case among direct readings, Severity 8 applies.</t>
         </is>
       </c>
       <c r="AQ18" s="223" t="inlineStr">
@@ -2554,23 +3028,35 @@
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>A = Add a machine‑vision inspection with controlled lighting to detect lens scratches and interlock the station to automatically reject discrepant headlamps.
-B = Add an in-station automated functional illumination test that powers the headlamp and measures current and lux with go/no-go limits to catch 'does not turn ON' and 'dim' before release.</t>
+          <t>A = Add an automated vision inspection gate for lens surface scratches that rejects/segregates discrepant headlamps before they leave the station or cell.
+-&gt; if adopted: D4 (Machine-based automated detection downstream that prevents outflow of discrepant product (D4).)
+B = Add an automated in‑station headlamp functional test that powers the unit and measures light output/current with a sensor, interlocked to stop transfer on fail.
+-&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing or routes to reject (D3).)</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible mechanism instead: apply a removable protective film to the headlamp lens from storage through installation, with a poka‑yoke removal step at final inspection to prevent handling scratches.
-B = The plant's recorded Cause does not match this Mode; addressing the more plausible damage mechanism instead: add a padded alignment/installation fixture with hard locating stops to support the headlamp and prevent lens/housing contact with the BIW during fitment and tightening.</t>
+          <t>A = The plant's recorded Cause does not match this Mode; addressing the likely scratch mechanism instead: add a protective film/cap on the lens and soft-lined guides/separators on the sequencing trolley and fixture contact points to prevent lens contact during handling and installation.
+B = The plant’s recorded Cause does not match this Mode; addressing the more plausible mechanism for DAMAGE instead: add a dedicated foam‑lined positioning fixture with locator pins to support the headlamp and prevent lens/edge contact during alignment and bolt‑tightening.</t>
         </is>
       </c>
       <c r="AT18" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage; it reads like the cause for a wrong-variant-installed row instead. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
+          <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
+- Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage Mode; it reads like the cause for a 'wrong variant installed' row instead.
+- Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing.
+- AI severity (8) differs from plant-recorded (5) - review recommended.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
  WRONG SELECTION OF HEAD LAMP
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
+      <c r="AU18" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect; Vague: Current Detection Controls</t>
+        </is>
+      </c>
+      <c r="AV18" s="223" t="inlineStr"/>
     </row>
     <row r="19" ht="207" customFormat="1" customHeight="1" s="8">
       <c r="B19" s="210" t="n"/>
@@ -2623,8 +3109,10 @@
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
       <c r="AT19" s="223" t="n"/>
-    </row>
-    <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
+      <c r="AU19" s="223" t="n"/>
+      <c r="AV19" s="223" t="n"/>
+    </row>
+    <row r="20" ht="127.5" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
       <c r="C20" s="211" t="n"/>
       <c r="D20" s="210" t="n"/>
@@ -2679,8 +3167,8 @@
       </c>
       <c r="AO20" s="223" t="inlineStr">
         <is>
-          <t>A = The End User effects explicitly state loss or degradation of the headlamp’s primary function (no illumination or dim light). This maps to loss of primary vehicle function (S=8) or degradation of primary function (S=7). Given both are equally plausible for a wrong-part selection, the worst applicable severity is 8.
-B = The listed End User effects for a wrong headlamp selection include both non-operation and dim output, which correspond to total loss or degradation of the headlamp’s primary function; there is no explicit safety or regulatory language, so severity is set by primary-function loss (worst-case S=8).</t>
+          <t>A = The End User effects include "Headlamp does not turn ON", which is a total loss of the primary lighting function used for normal driving; this maps to Severity 8. The alternative direct effect "dim light" would be Severity 7, but the worst equally representative direct case governs.
+B = The End User effects explicitly describe loss or degradation of the headlamp’s primary function; under the AIAG-VDA table, total loss maps to 8 and degradation to 7. With equal plausibility of both outcomes for a wrong-part selection, the worst-case 8 is used.</t>
         </is>
       </c>
       <c r="AQ20" s="223" t="inlineStr">
@@ -2691,21 +3179,32 @@
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>A = Use an in-station DC torque tool with transducer and PLC OK/NOK lockout to verify 6 Nm on each headlamp fastener and prevent release if torque is not achieved (detecting non-firm fitment).
-B = Implement an automated in-station headlamp functional test that powers the lamp after connection and measures current/illumination with sensors, stopping the line and flagging a mismatch if the unit is off or out of spec.</t>
+          <t>A = Add an automated, interlocked headlamp functional test at this station (command ON and verify current/illumination) that stops the station or routes to reject on fail.
+-&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing or automatically diverts to reject (D3).)
+B = Add an in-station barcode scan of the headlamp label validated against the vehicle’s BOM with a hard interlock that prevents OK-to-move/bolt-tightening on any mismatch.
+-&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing (D3).)</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
         <is>
-          <t>A = Add a VIN-driven pick-to-light/scan-interlocked sequencing trolley that only enables the correct headlamp bin for the build and alarms/locks the process if any other bin is accessed to prevent wrong-part picks.
-B = Add a barcode/RFID scan interlock tied to the build manifest that only enables the torque tool and allows installation when the scanned headlamp part number matches the vehicle model at this station.</t>
+          <t>A = Interlock the in-station part scan to the build manifest so that tool enable/OK-to-continue is blocked unless the scanned headlamp PN matches the VIN/sequence (prevents wrong-part installation).
+B = Implement a pick-to-light rack with model/VIN-linked bin locks so only the correct headlamp bin unlocks and others remain physically blocked at pick.</t>
         </is>
       </c>
       <c r="AT20" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing. AI severity (8) differs from plant-recorded (5) - review recommended. Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
-        </is>
-      </c>
+          <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
+- Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing.
+- AI severity (8) differs from plant-recorded (5) - review recommended.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+        </is>
+      </c>
+      <c r="AU20" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect; Vague: Current Detection Controls</t>
+        </is>
+      </c>
+      <c r="AV20" s="223" t="inlineStr"/>
     </row>
     <row r="21" ht="153" customFormat="1" customHeight="1" s="8">
       <c r="B21" s="210" t="n"/>
@@ -2758,6 +3257,8 @@
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
       <c r="AT21" s="223" t="n"/>
+      <c r="AU21" s="223" t="n"/>
+      <c r="AV21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2777,16 +3278,82 @@
       <c r="L22" s="210" t="n"/>
       <c r="M22" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wiring harness partially connected (loose fitment)
 2. Electrical connector loose or damaged
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Incorrect beam alignment
 2. Headlamp does not turn ON
 3. Reduced road visibility
 4. Increased risk of accident</t>
+          </r>
         </is>
       </c>
       <c r="N22" s="207" t="n"/>
@@ -2827,7 +3394,7 @@
       </c>
       <c r="AO22" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly list 'Increased risk of accident', which is causally plausible for an unconnected/poorly locked headlamp connector causing the lamp not to turn on and reducing visibility. Per the table, this is a safety/health risk to road users, so Severity is 10.</t>
+          <t>The End User effects explicitly include “Increased risk of accident,” which is a plausible consequence of a headlamp not turning on due to an improperly locked/forgotten connector, so this meets the safety/health risk criterion.</t>
         </is>
       </c>
       <c r="AQ22" s="223" t="n">
@@ -2835,19 +3402,26 @@
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Add an in‑station automated functional test that powers each headlamp and verifies illumination/current draw with a light or current sensor, stopping the process if either lamp fails.</t>
+          <t>Install an in-station automated electrical continuity/illumination test for both headlamp circuits with interlock to stop the process or reject the unit if either lamp is not powered.
+-&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing/outflow (D3).)</t>
         </is>
       </c>
       <c r="AS22" s="223" t="inlineStr">
         <is>
-          <t>Add a connector-lock poka‑yoke: a mechanical go/no‑go gauge or latch‑position sensor interlocked with the station PLC so the cycle cannot complete unless the connector latch is fully engaged.</t>
+          <t>Add a connector position assurance (CPA) secondary lock to the headlamp connectors so incomplete or forgotten mating is physically prevented.</t>
         </is>
       </c>
       <c r="AT22" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
-        </is>
-      </c>
+          <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+        </is>
+      </c>
+      <c r="AU22" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect</t>
+        </is>
+      </c>
+      <c r="AV22" s="223" t="inlineStr"/>
     </row>
     <row r="23" ht="186.95" customFormat="1" customHeight="1" s="14">
       <c r="B23" s="210" t="n"/>
@@ -2920,6 +3494,8 @@
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
       <c r="AT23" s="223" t="n"/>
+      <c r="AU23" s="223" t="n"/>
+      <c r="AV23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -2978,7 +3554,7 @@
       </c>
       <c r="AO24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly state 'Increased risk of accident,' which is a plausible consequence of an unbolted/misaligned headlamp causing reduced road illumination. Per the scoring rules and Table C2-1, this constitutes an effect that affects safe operation of the vehicle, warranting Severity 10.</t>
+          <t>The End User effects explicitly include "Increased risk of accident," which plausibly results from an unbolted/misaligned headlamp reducing forward illumination. Per the table, that is a safety/health-risk impact to the end user, warranting Severity 10.</t>
         </is>
       </c>
       <c r="AQ24" s="223" t="n">
@@ -2986,19 +3562,26 @@
       </c>
       <c r="AR24" s="223" t="inlineStr">
         <is>
-          <t>Install a machine-vision presence/position check at station exit to verify both headlamp bolt heads are present and seated, with automatic NOK stop/reject if either bolt is missing.</t>
+          <t>Install an in-station torque/angle controller with per-bolt count and OK/NOK line interlock to detect any missed or not-torqued headlamp prefit bolts before release.
+-&gt; if adopted: D3 (Machine-based, in-station, stops further processing (D3))</t>
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr">
         <is>
-          <t>Add a DC electric nutrunner with torque/angle monitoring and an OK-to-proceed interlock that requires both headlamp bolts to be run to 6 Nm (correct count and torque achieved) before allowing the station to complete.</t>
+          <t>Implement pick-to-light kitting with photoelectric sensors for the required headlamp bolts, interlocked so the job cannot start/advance until all bolts are picked for install.</t>
         </is>
       </c>
       <c r="AT24" s="223" t="inlineStr">
         <is>
-          <t>AI severity (10) differs from plant-recorded (5) - review recommended.</t>
-        </is>
-      </c>
+          <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
+        </is>
+      </c>
+      <c r="AU24" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect; Vague: Failure Cause</t>
+        </is>
+      </c>
+      <c r="AV24" s="223" t="inlineStr"/>
     </row>
     <row r="25" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B25" s="210" t="n"/>
@@ -3055,6 +3638,8 @@
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
       <c r="AT25" s="223" t="n"/>
+      <c r="AU25" s="223" t="n"/>
+      <c r="AV25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3074,16 +3659,103 @@
       <c r="L26" s="210" t="n"/>
       <c r="M26" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting screws under-torqued or over-torqued
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Lens cracked or broken
 2. LED / BULB burnout
 3. Water ingress inside lamp
 4. Rattling or vibration noise during driving
 5. Driver discomfort or eye strain</t>
+          </r>
         </is>
       </c>
       <c r="N26" s="207" t="n"/>
@@ -3129,8 +3801,8 @@
       </c>
       <c r="AO26" s="223" t="inlineStr">
         <is>
-          <t>A = The direct customer-facing consequence of failing to fit the mounting screws is a loose lamp causing rattling/vibration noise during driving, which aligns with a very objectionable NVH condition per the table.
-B = Among the listed End User effects, water ingress is the direct consequence of an uneven headlamp-to-fender gap and is best characterized as a very objectionable visible condition to the customer; no explicit safety, regulatory, or stated primary-function loss is given.</t>
+          <t>A = The most direct End User outcome of failed-to-fit screws from uneven gaps is "rattling or vibration noise during driving," which maps to very objectionable NVH. No explicit safety or regulatory effect is stated for this row, and other listed outcomes require additional unstated mechanisms.
+B = The DIRECT end-user outcome of this gap/flushness error is rattling/vibration noise while driving, which is an NVH complaint. No accident/injury or regulatory consequence is stated, and the primary lighting function is not directly impacted for this Mode/Cause.</t>
         </is>
       </c>
       <c r="AQ26" s="223" t="inlineStr">
@@ -3141,21 +3813,31 @@
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>A = Use an electronic torque controller that counts each fastener and verifies torque/angle OK for all required screws, blocking proceed on any missing/under/over-torqued condition.
-B = Install an in-station camera-based gap/flushness measurement system interlocked to the station (block OK-to-release if any measured gap/flushness is out of spec).</t>
+          <t>A = Use an EC-nutrunner with torque/angle/rundown monitoring and fastener count OK/NOK interlock that blocks station completion unless each headlamp screw reaches 6 Nm within angle window.
+-&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
+B = Add an in-station machine-vision gap/flushness measurement with interlock that prevents proceeding unless gap/flushness at defined points is within specification.
+-&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>A = Add a datum-based alignment/locator fixture with hard edge stops and hole locators to set the headlamp-to-fender gap and align the screw bosses before fastening so screws can be fitted correctly every time.
-B = Add a dedicated locating/positioning fixture or hard datum pins at the headlamp mounting points to set flushness and gap to spec before torquing, preventing misalignment by design.</t>
+          <t>A = Add a dedicated headlamp locating fixture with BIW datum hard-stops/dowel pins to set uniform fender gaps before fastening so the screw holes align and cross-threading/failed fit cannot occur.
+B = Introduce a simple 3-point gap/flushness locator fixture or go/no-go gap shims to hold the headlamp to the specified gaps against the fender/BIW while bolts are torqued to 6 Nm.</t>
         </is>
       </c>
       <c r="AT26" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Cause/Mode mismatch: The recorded Cause addresses only gap uniformity between headlamp edge and fender and does not explain the merged Mode’s "failed to fit screws" sub-mode.</t>
-        </is>
-      </c>
+          <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
+- Cause/Mode mismatch: The stated Cause addresses only non-uniform gaps, not the 'failed to fit screws' portion of the Mode.</t>
+        </is>
+      </c>
+      <c r="AU26" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
+      <c r="AV26" s="223" t="inlineStr"/>
     </row>
     <row r="27" ht="156" customFormat="1" customHeight="1" s="13">
       <c r="B27" s="210" t="n"/>
@@ -3218,6 +3900,8 @@
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
       <c r="AT27" s="223" t="n"/>
+      <c r="AU27" s="223" t="n"/>
+      <c r="AV27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3289,29 +3973,37 @@
       </c>
       <c r="AO28" s="223" t="inlineStr">
         <is>
-          <t>The only direct customer effect of an under-torqued headlamp mounting is rattling/vibration noise while driving, which is an NVH issue. The list contains no explicit safety or regulatory consequence tied to this mode, so severity aligns with "very objectionable" NVH at S=4.</t>
+          <t>For an under-torqued headlamp mount, the DIRECT end-user outcome listed is rattling/vibration noise while driving, which maps to very objectionable NVH. No explicit safety or regulatory consequence is stated, and other listed effects require additional, unstated failure steps.</t>
         </is>
       </c>
       <c r="AQ28" s="223" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AR28" s="223" t="inlineStr">
         <is>
-          <t>Install a transducerized DC nutrunner or in-line torque/angle monitor that records actual achieved torque and provides OK/NOK with line stop if 6 Nm is not reached.</t>
+          <t>Add in-station torque transducer monitoring with the nutrunner controller that records OK/NOK per bolt and stops the station or prevents advancement on any NOK torque.
+-&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr">
         <is>
-          <t>Add a station interlock with tool-ID/torque-program lock (RFID/barcode pairing) so only the correct, calibrated 6 Nm power tool can run this joint and its torque setting cannot be changed by the operator.</t>
+          <t>Install a controller-based DC nutrunner for the headlamp bolts with program-locked 6 Nm, socket/tool ID verification, bolt-count, and OK/NOK interlock to prevent job completion unless torque is achieved.</t>
         </is>
       </c>
       <c r="AT28" s="223" t="inlineStr">
         <is>
-          <t>Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="118.5" customFormat="1" customHeight="1" s="13">
+          <t>- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+        </is>
+      </c>
+      <c r="AU28" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
+      <c r="AV28" s="223" t="inlineStr"/>
+    </row>
+    <row r="29" ht="240" customFormat="1" customHeight="1" s="13">
       <c r="B29" s="210" t="n"/>
       <c r="C29" s="211" t="n"/>
       <c r="D29" s="210" t="n"/>
@@ -3352,49 +4044,59 @@
       <c r="AL29" s="10" t="n"/>
       <c r="AM29" s="223" t="inlineStr">
         <is>
-          <t>A = Torque not achieved
-B = Over torque</t>
+          <t>A = Under-torque (torque not achieved)
+B = Over-torque</t>
         </is>
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
           <t>A = 4
-B = 4</t>
+B = 7</t>
         </is>
       </c>
       <c r="AO29" s="223" t="inlineStr">
         <is>
-          <t>A = For this torque error, the direct user-facing outcomes are either a cracked/broken lens (over‑torque) or rattling/vibration noise (under‑torque), both of which fit the table’s “very objectionable appearance/sound/vibration/harshness/haptics” definition; no safety, regulatory, or explicit primary-function loss is stated.
-B = The DIRECT End User effect of over‑torque here is a cracked/broken lens, which is best characterized as a very objectionable appearance defect; the other listed effects (burnout, water ingress, rattling, discomfort) require additional unstated steps and are therefore INDIRECT.</t>
+          <t>A = For under-torque of the headlamp mounting, the only direct end-user effect listed is rattling/vibration during driving, which is an NVH complaint. Per the table, objectionable noise/vibration maps to Severity 4. Other listed effects (crack, burnout, water ingress, eye strain) require additional unstated failure steps and are indirect for this mode/cause.
+B = The direct end user effect of over‑torque is a cracked/broken lens, which would degrade headlamp performance rather than eliminate it entirely. No accident/injury or regulatory language is stated, so this aligns with degraded primary function.</t>
         </is>
       </c>
       <c r="AQ29" s="223" t="inlineStr">
         <is>
-          <t>A = 9
+          <t>A = 8
 B = 9</t>
         </is>
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>A = Integrate in‑station torque monitoring (nutrunner torque‑angle OK/NOK with PLC interlock) so the station cannot advance unless each fastener achieves the 6 Nm OK result.
-B = Integrate in‑station electronic torque monitoring with data logging and an interlock that blocks job release if the recorded torque is outside the 6 Nm window (OK/NOK confirmation).</t>
+          <t>A = Install a controller-monitored DC nutrunner with torque/angle monitoring and OK/NOK interlock that prevents station completion if 6 Nm is not achieved.
+-&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
+B = Add in‑station torque/angle monitoring with automatic NOK lockout that stops processing if any headlamp fastener exceeds the upper torque limit.
+-&gt; if adopted: D2 (Machine-based detection method that will detect the CAUSE and PREVENT the failure mode (discrepant part) from being produced (D2).)</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>A = Install a DC electric nutrunner with controller‑locked 6 Nm program and RFID/tool‑ID lockout so the station cannot run with the wrong tool or setting, directly addressing operator mistake and wrong/miscalibrated tool causes.
-B = Install a DC torque-controlled driver locked to a 6 Nm window with OK/NOK lockout (paired to this station/tool ID) to prevent over‑torque from operator error, wrong tool use, or drift.</t>
+          <t>A = Add a tool-ID and calibration-status interlock tied to part scan so only the correct, in-calibration 6 Nm DC nutrunner can run this operation and all other tools are locked out.
+B = Replace the labeled dedicated gun with a transducerized shut‑off torque tool programmed to 6 Nm with an upper torque limit and PLC interlock that blocks the cycle on NOK/tool‑mismatch and logs torque results.</t>
         </is>
       </c>
       <c r="AT29" s="223" t="inlineStr">
         <is>
-          <t>Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text. Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
-        </is>
-      </c>
+          <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
+- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
+        </is>
+      </c>
+      <c r="AU29" s="223" t="inlineStr">
+        <is>
+          <t>- Missing: Ship-to-Plant effect
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
+      <c r="AV29" s="223" t="inlineStr"/>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="181">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
@@ -3402,6 +4104,7 @@
     <mergeCell ref="AM15:AM17"/>
     <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
+    <mergeCell ref="AV18:AV19"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
@@ -3412,18 +4115,20 @@
     <mergeCell ref="T13:AA14"/>
     <mergeCell ref="S1:T2"/>
     <mergeCell ref="D12:F12"/>
+    <mergeCell ref="AU24:AU25"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G13:L14"/>
     <mergeCell ref="AR24:AR25"/>
     <mergeCell ref="K9:T9"/>
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
+    <mergeCell ref="AU26:AU27"/>
     <mergeCell ref="AN15:AN17"/>
     <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
-    <mergeCell ref="AM13:AT14"/>
+    <mergeCell ref="AU18:AU19"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3443,7 +4148,9 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
+    <mergeCell ref="AM13:AV14"/>
     <mergeCell ref="AT15:AT17"/>
+    <mergeCell ref="AV15:AV17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
@@ -3477,6 +4184,7 @@
     <mergeCell ref="AC15:AC17"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
+    <mergeCell ref="AV20:AV21"/>
     <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AS24:AS25"/>
     <mergeCell ref="AD15:AD17"/>
@@ -3488,6 +4196,8 @@
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
     <mergeCell ref="AS20:AS21"/>
+    <mergeCell ref="AU20:AU21"/>
+    <mergeCell ref="AV22:AV23"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
@@ -3509,13 +4219,16 @@
     <mergeCell ref="AM20:AM21"/>
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
+    <mergeCell ref="AV24:AV25"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="AO22:AO23"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
     <mergeCell ref="AT22:AT23"/>
+    <mergeCell ref="AV26:AV27"/>
     <mergeCell ref="T19:U19"/>
+    <mergeCell ref="AU15:AU17"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
@@ -3561,6 +4274,7 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="AU22:AU23"/>
     <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>
@@ -4056,9 +4770,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -4077,8 +4813,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -4299,37 +5057,294 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 FRONT GRILL FITMENT- HIGH VARIANT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Connections, 
 Bolts &amp; pushpin   fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 To correctly install front grill fitment as per BIW design specifications.
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Allow airflow to the radiator, condenser, and engine compartment
 2. Protect cooling components from debris, stones, insects
 3. Provide vehicle styling and brand identity</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -4341,33 +5356,186 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. TAKE THE FRONT GRILL FROM THE STORAGE AREA AND SCAN THE PART
 2. CONNECT THE CONNECTORS WITH GRILL
 3. INSERT &amp; 
 ALIGN THE FRONT GRILL WITH BIW AND THEN TIGHT WITH BOLTS AND PUSHPINS
-2. Machine:
-Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Front grill from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Front grill from sequencing trolley and scan
 2. Then do the connections with wiring harness with grill and align with BIW and tight with bolts &amp; pushpins
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong front grill variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Gaps or scratches on grill 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Incorrect distance / object detection
 2. Water/dust ingress affecting sensor
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -4565,16 +5733,82 @@
       <c r="L22" s="210" t="n"/>
       <c r="M22" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wiring harness partially connected (loose fitment)
 2. Wiring harness pinched or damaged
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. False ADAS warnings or alerts
 2. Incorrect object detection
 3. Lane assist / collision warning inoperative
 4. Increased risk of accident</t>
+          </r>
         </is>
       </c>
       <c r="N22" s="207" t="n"/>
@@ -4781,16 +6015,103 @@
       <c r="L26" s="210" t="n"/>
       <c r="M26" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting bolts under-torqued or over-torqued
 3. Broken clips
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Customer loss of confidence in vehicle safety
 2. False collision warnings provided to driver
 3. Water/dust ingress affecting sensor
 4. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N26" s="207" t="n"/>
@@ -5592,9 +6913,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -5613,8 +6956,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -5835,36 +7200,293 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 FRONT GRILL FITMENT- LOW VARIANT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Bolts &amp; pushpin   fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 To correctly install front grill fitment as per BIW design specifications.
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Allow airflow to the radiator, condenser, and engine compartment
 2. Protect cooling components from debris, stones, insects
 3. Provide vehicle styling and brand identity</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -5876,32 +7498,185 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. TAKE THE FRONT GRILL FROM THE STORAGE AREA AND SCAN THE PART
 2. INSERT &amp; 
 ALIGN THE FRONT GRILL WITH BIW AND THEN TIGHT WITH BOLTS AND PUSHPINS
-2. Machine:
-Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Front grill from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Front grill from sequencing trolley and scan
 2. Align with BIW and tight with bolts &amp; pushpins
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong front grill variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Gaps or scratches on grill 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting sensor
 2. Customer dissatisfaction
 3. Bad appereance of vehicle</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -6062,11 +7837,77 @@
       <c r="L21" s="210" t="n"/>
       <c r="M21" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting part warrenty</t>
+          </r>
         </is>
       </c>
       <c r="N21" s="207" t="n"/>
@@ -6242,14 +8083,101 @@
       <c r="L24" s="210" t="n"/>
       <c r="M24" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting bolts under-torqued or over-torqued
 3. Broken clips
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting sensor
 2. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N24" s="207" t="n"/>
@@ -7063,9 +8991,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -7084,8 +9034,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -7306,37 +9278,294 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 LH / RH RADIATOR SIDE SEAL FITMENT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Screw &amp; pushpin fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Correct installation and positioning of the side seal during radiator assembly.
 2. Maintain seal integrity (no cuts, twists or misalignment)
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Maintain system pressure under operating temperature and vibration
 2. Accommodate thermal expansion between radiator components
 3. Seal the joint between the radiator core and side tank to prevent coolant leakage</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -7348,30 +9577,183 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. GET THE SIDE SEAL FROM STORAGE BIN
 2. ALIGN THE SIDE SEAL WITH THE BIW AND THEN TIGHT WITH BOLT AND PUSHPIN
-2. Machine:
-Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Take side seal from storage bin
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Take side seal from storage bin
 2. Align side seal with BIW and tight with bolt and pushpin
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong part installed or mixed material
 2. FURTHER OPERATION NOT POSSIBLE
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Vehicle overheating
 2. Coolant seepage or visible leak
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -7480,15 +9862,81 @@
       <c r="L20" s="210" t="n"/>
       <c r="M20" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Cut, torn, pinched, or cracked seal
 2. Seal under-compressed or over-compressed
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Reduced cooling efficiency
 2. Engine overheating
 3. Safety risk if overheating occurs during driving</t>
+          </r>
         </is>
       </c>
       <c r="N20" s="207" t="n"/>
@@ -7757,14 +10205,101 @@
       <c r="L25" s="210" t="n"/>
       <c r="M25" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting Bolt under-torqued or over-torqued
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Customer dissatisfaction due to coolant leak
 2. Coolant dripping under vehicle
 3. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N25" s="207" t="n"/>

</xml_diff>

<commit_message>
Rebuild merge-mode Excel: readable Detection projection + sanitized cells
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -3029,9 +3029,9 @@
       <c r="AR18" s="223" t="inlineStr">
         <is>
           <t>A = Add an automated vision inspection gate for lens surface scratches that rejects/segregates discrepant headlamps before they leave the station or cell.
--&gt; if adopted: D4 (Machine-based automated detection downstream that prevents outflow of discrepant product (D4).)
+If adopted, Detection = 4 (Machine-based automated detection downstream that prevents outflow of discrepant product (D4).)
 B = Add an automated in‑station headlamp functional test that powers the unit and measures light output/current with a sensor, interlocked to stop transfer on fail.
--&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing or routes to reject (D3).)</t>
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing or routes to reject (D3).)</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
@@ -3180,9 +3180,9 @@
       <c r="AR20" s="223" t="inlineStr">
         <is>
           <t>A = Add an automated, interlocked headlamp functional test at this station (command ON and verify current/illumination) that stops the station or routes to reject on fail.
--&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing or automatically diverts to reject (D3).)
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing or automatically diverts to reject (D3).)
 B = Add an in-station barcode scan of the headlamp label validated against the vehicle’s BOM with a hard interlock that prevents OK-to-move/bolt-tightening on any mismatch.
--&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing (D3).)</t>
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing (D3).)</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
@@ -3403,7 +3403,7 @@
       <c r="AR22" s="223" t="inlineStr">
         <is>
           <t>Install an in-station automated electrical continuity/illumination test for both headlamp circuits with interlock to stop the process or reject the unit if either lamp is not powered.
--&gt; if adopted: D3 (Machine-based automated detection in-station that prevents further processing/outflow (D3).)</t>
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing/outflow (D3).)</t>
         </is>
       </c>
       <c r="AS22" s="223" t="inlineStr">
@@ -3563,7 +3563,7 @@
       <c r="AR24" s="223" t="inlineStr">
         <is>
           <t>Install an in-station torque/angle controller with per-bolt count and OK/NOK line interlock to detect any missed or not-torqued headlamp prefit bolts before release.
--&gt; if adopted: D3 (Machine-based, in-station, stops further processing (D3))</t>
+If adopted, Detection = 3 (Machine-based, in-station, stops further processing (D3))</t>
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr">
@@ -3814,9 +3814,9 @@
       <c r="AR26" s="223" t="inlineStr">
         <is>
           <t>A = Use an EC-nutrunner with torque/angle/rundown monitoring and fastener count OK/NOK interlock that blocks station completion unless each headlamp screw reaches 6 Nm within angle window.
--&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
 B = Add an in-station machine-vision gap/flushness measurement with interlock that prevents proceeding unless gap/flushness at defined points is within specification.
--&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
@@ -3982,7 +3982,7 @@
       <c r="AR28" s="223" t="inlineStr">
         <is>
           <t>Add in-station torque transducer monitoring with the nutrunner controller that records OK/NOK per bolt and stops the station or prevents advancement on any NOK torque.
--&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr">
@@ -4069,9 +4069,9 @@
       <c r="AR29" s="223" t="inlineStr">
         <is>
           <t>A = Install a controller-monitored DC nutrunner with torque/angle monitoring and OK/NOK interlock that prevents station completion if 6 Nm is not achieved.
--&gt; if adopted: D3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
 B = Add in‑station torque/angle monitoring with automatic NOK lockout that stops processing if any headlamp fastener exceeds the upper torque limit.
--&gt; if adopted: D2 (Machine-based detection method that will detect the CAUSE and PREVENT the failure mode (discrepant part) from being produced (D2).)</t>
+If adopted, Detection = 2 (Machine-based detection method that will detect the CAUSE and PREVENT the failure mode (discrepant part) from being produced (D2).)</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild merge-mode Excel: clean Detection projection note (no nested D-score)
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode.xlsx
@@ -2472,7 +2472,7 @@
       <c r="AU17" s="208" t="n"/>
       <c r="AV17" s="208" t="n"/>
     </row>
-    <row r="18" ht="142.5" customFormat="1" customHeight="1" s="8">
+    <row r="18" ht="150" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
         <is>
           <t>HEAD LAMP STAGE</t>
@@ -3005,19 +3005,19 @@
       <c r="AM18" s="223" t="inlineStr">
         <is>
           <t>A = SCRATCH
-B = DAMAGE</t>
+B = DAMAGE ON HEAD LAMP</t>
         </is>
       </c>
       <c r="AN18" s="223" t="inlineStr">
         <is>
-          <t>A = 7
+          <t>A = 3
 B = 8</t>
         </is>
       </c>
       <c r="AO18" s="223" t="inlineStr">
         <is>
-          <t>A = Among the listed End User effects, a scratched headlamp lens most directly leads to "Insufficient brightness / dim light", which is a degradation of the primary lighting function. No explicit safety or regulatory language is stated, and "does not turn on" would require an additional electrical fault not described for a scratch.
-B = The End User effects include "Headlamp does not turn ON" (total loss of the headlamp’s primary function) and "Insufficient brightness / dim light" (degradation). With the Mode "DAMAGE" unspecified, both are plausible direct outcomes; per the worst-case among direct readings, Severity 8 applies.</t>
+          <t>A = The representative End User effect for a scratch is a cosmetic complaint (customer dissatisfaction), which maps to the table’s appearance/haptics category at the end user. No accident/injury or regulatory wording is present, and the primary lighting function is not claimed lost for this mode.
+B = End User effects list both 'does not turn ON' and 'dim light' for a damaged headlamp, which map to loss vs degradation of the primary lighting function; with no explicit safety or regulatory wording, the worst applicable is loss of primary function (8).</t>
         </is>
       </c>
       <c r="AQ18" s="223" t="inlineStr">
@@ -3028,22 +3028,22 @@
       </c>
       <c r="AR18" s="223" t="inlineStr">
         <is>
-          <t>A = Add an automated vision inspection gate for lens surface scratches that rejects/segregates discrepant headlamps before they leave the station or cell.
-If adopted, Detection = 4 (Machine-based automated detection downstream that prevents outflow of discrepant product (D4).)
-B = Add an automated in‑station headlamp functional test that powers the unit and measures light output/current with a sensor, interlocked to stop transfer on fail.
-If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing or routes to reject (D3).)</t>
+          <t>A = Add an in-station automated vision inspection to check the headlamp lens surface for scratches after installation and interlock to route any discrepant unit to a reject lane.
+If adopted, Detection = 3 (Machine-based automated detection in-station that detects the failure mode and prevents further processing or routes automatically to a reject area)
+B = Add an in-station automated headlamp functional test that powers the lamp and measures light intensity/ON status with a sensor, interlocking the station on fail.
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing, a robust system that prevents outflow.)</t>
         </is>
       </c>
       <c r="AS18" s="223" t="inlineStr">
         <is>
-          <t>A = The plant's recorded Cause does not match this Mode; addressing the likely scratch mechanism instead: add a protective film/cap on the lens and soft-lined guides/separators on the sequencing trolley and fixture contact points to prevent lens contact during handling and installation.
-B = The plant’s recorded Cause does not match this Mode; addressing the more plausible mechanism for DAMAGE instead: add a dedicated foam‑lined positioning fixture with locator pins to support the headlamp and prevent lens/edge contact during alignment and bolt‑tightening.</t>
+          <t>A = The plant's recorded Cause does not match this Mode; addressing the more plausible scratch mechanism instead: apply a removable protective film/cover on the headlamp lens through handling and installation, with a defined removal step after fitment.
+B = The plant's recorded Cause does not match this Mode; addressing damage mechanisms instead: add a snap-on protective lens cover and foam-lined, dedicated slots on the sequencing trolley to prevent lens/contact damage during handling and installation.</t>
         </is>
       </c>
       <c r="AT18" s="223" t="inlineStr">
         <is>
           <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
-- Cause/Mode mismatch: This Cause (wrong part selection/mix-up) does not produce a scratch/damage Mode; it reads like the cause for a 'wrong variant installed' row instead.
+- Cause/Mode mismatch: This Cause (wrong part/mix-up) does not produce a scratch/damage mode; it aligns more with a 'wrong variant installed' failure instead.
 - Ambiguous - plausible severities: S8 (Headlamp does not turn ON); S7 (Insufficient brightness / dim light). Suggested value is the worst case; review before finalizing.
 - AI severity (8) differs from plant-recorded (5) - review recommended.
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: FITMENT IS NOT FIRM
@@ -3053,7 +3053,7 @@
       </c>
       <c r="AU18" s="223" t="inlineStr">
         <is>
-          <t>- Missing: Ship-to-Plant effect; Vague: Current Detection Controls</t>
+          <t>- Missing: Ship-to-Plant effect; Vague: Detection Controls</t>
         </is>
       </c>
       <c r="AV18" s="223" t="inlineStr"/>
@@ -3112,7 +3112,7 @@
       <c r="AU19" s="223" t="n"/>
       <c r="AV19" s="223" t="n"/>
     </row>
-    <row r="20" ht="127.5" customFormat="1" customHeight="1" s="8">
+    <row r="20" ht="142.5" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
       <c r="C20" s="211" t="n"/>
       <c r="D20" s="210" t="n"/>
@@ -3156,7 +3156,7 @@
       <c r="AM20" s="223" t="inlineStr">
         <is>
           <t>A = Fitment is not firm
-B = Wrong selection of headlamp (not as per model)</t>
+B = Wrong selection of head lamp (not as per model)</t>
         </is>
       </c>
       <c r="AN20" s="223" t="inlineStr">
@@ -3167,8 +3167,8 @@
       </c>
       <c r="AO20" s="223" t="inlineStr">
         <is>
-          <t>A = The End User effects include "Headlamp does not turn ON", which is a total loss of the primary lighting function used for normal driving; this maps to Severity 8. The alternative direct effect "dim light" would be Severity 7, but the worst equally representative direct case governs.
-B = The End User effects explicitly describe loss or degradation of the headlamp’s primary function; under the AIAG-VDA table, total loss maps to 8 and degradation to 7. With equal plausibility of both outcomes for a wrong-part selection, the worst-case 8 is used.</t>
+          <t>A = The End User effects list includes "Headlamp does not turn ON", which is a loss of the headlamp’s primary function; per the table this maps to Severity 8.
+B = The End User effects list total loss of illumination and degraded illumination, both tied directly to installing the wrong headlamp variant; these map to loss/degradation of a primary vehicle function. No explicit safety or regulatory wording is present, so the worst applicable Step 3 definition (8) applies.</t>
         </is>
       </c>
       <c r="AQ20" s="223" t="inlineStr">
@@ -3179,16 +3179,16 @@
       </c>
       <c r="AR20" s="223" t="inlineStr">
         <is>
-          <t>A = Add an automated, interlocked headlamp functional test at this station (command ON and verify current/illumination) that stops the station or routes to reject on fail.
-If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing or automatically diverts to reject (D3).)
-B = Add an in-station barcode scan of the headlamp label validated against the vehicle’s BOM with a hard interlock that prevents OK-to-move/bolt-tightening on any mismatch.
-If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing (D3).)</t>
+          <t>A = Install an automated in-station headlamp functional test that powers the unit and measures current/illumination, interlocked to stop/reject if either side fails.
+If adopted, Detection = 3 (Machine-based automated detection in-station that will detect the failure mode and prevent further processing/outflow)
+B = Install an automated in-station functional headlamp test that powers the lamp and measures lux with a calibrated sensor, rejecting and stopping the station on out-of-spec or no-light conditions.
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing, robustly preventing outflow.)</t>
         </is>
       </c>
       <c r="AS20" s="223" t="inlineStr">
         <is>
-          <t>A = Interlock the in-station part scan to the build manifest so that tool enable/OK-to-continue is blocked unless the scanned headlamp PN matches the VIN/sequence (prevents wrong-part installation).
-B = Implement a pick-to-light rack with model/VIN-linked bin locks so only the correct headlamp bin unlocks and others remain physically blocked at pick.</t>
+          <t>A = Add MES-driven pick-to-light with bin locks on the sequencing trolley so only the correct LH/RH headlamp variant bin opens for the current VIN/build.
+B = Add a pick-to-light plus barcode/2D-code scan at the storage trolley interlocked to the build manifest so a non-matching headlamp cannot be picked or released to the station.</t>
         </is>
       </c>
       <c r="AT20" s="223" t="inlineStr">
@@ -3199,11 +3199,7 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AU20" s="223" t="inlineStr">
-        <is>
-          <t>- Missing: Ship-to-Plant effect; Vague: Current Detection Controls</t>
-        </is>
-      </c>
+      <c r="AU20" s="223" t="inlineStr"/>
       <c r="AV20" s="223" t="inlineStr"/>
     </row>
     <row r="21" ht="153" customFormat="1" customHeight="1" s="8">
@@ -3394,7 +3390,7 @@
       </c>
       <c r="AO22" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include “Increased risk of accident,” which is a plausible consequence of a headlamp not turning on due to an improperly locked/forgotten connector, so this meets the safety/health risk criterion.</t>
+          <t>The End User effects explicitly include “Increased risk of accident,” which is a plausible consequence of an unlatched/forgotten headlamp connector causing the lamp to not turn on and reducing road visibility. This affects safe operation of the vehicle, matching the Severity 10 definition.</t>
         </is>
       </c>
       <c r="AQ22" s="223" t="n">
@@ -3402,13 +3398,13 @@
       </c>
       <c r="AR22" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station automated electrical continuity/illumination test for both headlamp circuits with interlock to stop the process or reject the unit if either lamp is not powered.
-If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing/outflow (D3).)</t>
+          <t>Implement an automated in‑station functional test that commands low/high beam and measures current or illuminance, auto‑stopping and rejecting the unit if either beam does not meet thresholds.
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing; a robust system that prevents outflow of discrepant product.)</t>
         </is>
       </c>
       <c r="AS22" s="223" t="inlineStr">
         <is>
-          <t>Add a connector position assurance (CPA) secondary lock to the headlamp connectors so incomplete or forgotten mating is physically prevented.</t>
+          <t>Add a connector-latch poka‑yoke: a mechanical latch-sensing interlock on both headlamp connectors that prevents advancing/bolting until each connector is fully seated and locked.</t>
         </is>
       </c>
       <c r="AT22" s="223" t="inlineStr">
@@ -3416,11 +3412,7 @@
           <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
-      <c r="AU22" s="223" t="inlineStr">
-        <is>
-          <t>- Missing: Ship-to-Plant effect</t>
-        </is>
-      </c>
+      <c r="AU22" s="223" t="inlineStr"/>
       <c r="AV22" s="223" t="inlineStr"/>
     </row>
     <row r="23" ht="186.95" customFormat="1" customHeight="1" s="14">
@@ -3554,7 +3546,7 @@
       </c>
       <c r="AO24" s="223" t="inlineStr">
         <is>
-          <t>The End User effects explicitly include "Increased risk of accident," which plausibly results from an unbolted/misaligned headlamp reducing forward illumination. Per the table, that is a safety/health-risk impact to the end user, warranting Severity 10.</t>
+          <t>The End User effects explicitly include "Increased risk of accident" arising from a headlamp that may be misaligned or not functioning, which plausibly follows from bolts not being prefitted. Per the table, this is a safety/health risk to road users and affects safe operation of the vehicle.</t>
         </is>
       </c>
       <c r="AQ24" s="223" t="n">
@@ -3562,13 +3554,13 @@
       </c>
       <c r="AR24" s="223" t="inlineStr">
         <is>
-          <t>Install an in-station torque/angle controller with per-bolt count and OK/NOK line interlock to detect any missed or not-torqued headlamp prefit bolts before release.
-If adopted, Detection = 3 (Machine-based, in-station, stops further processing (D3))</t>
+          <t>Add in-station automated bolt presence and torque verification (DC nutrunners with OK/NOK and line stop) to detect any missing/untorqued headlamp bolts before the vehicle leaves the station.
+If adopted, Detection = 2 (Machine-based detection that will detect the cause and prevent the failure mode from being produced)</t>
         </is>
       </c>
       <c r="AS24" s="223" t="inlineStr">
         <is>
-          <t>Implement pick-to-light kitting with photoelectric sensors for the required headlamp bolts, interlocked so the job cannot start/advance until all bolts are picked for install.</t>
+          <t>Implement PLC-guided DC electric nutrunners with bolt-count and 6 Nm OK interlock so the station cannot be completed or advanced unless all required headlamp bolts are installed and torqued to spec.</t>
         </is>
       </c>
       <c r="AT24" s="223" t="inlineStr">
@@ -3801,8 +3793,8 @@
       </c>
       <c r="AO26" s="223" t="inlineStr">
         <is>
-          <t>A = The most direct End User outcome of failed-to-fit screws from uneven gaps is "rattling or vibration noise during driving," which maps to very objectionable NVH. No explicit safety or regulatory effect is stated for this row, and other listed outcomes require additional unstated mechanisms.
-B = The DIRECT end-user outcome of this gap/flushness error is rattling/vibration noise while driving, which is an NVH complaint. No accident/injury or regulatory consequence is stated, and the primary lighting function is not directly impacted for this Mode/Cause.</t>
+          <t>A = The direct End User symptom of loose/misfit screws is rattling/vibration noise while driving, which is an NVH complaint. Per the table, very objectionable sound/vibration maps to Severity 4. No explicit safety or regulatory consequence is stated for this row.
+B = The direct customer-facing consequence of non-uniform headlamp-to-fender gap is NVH (rattling/vibration noise) during driving, which aligns with the 'very objectionable' sound/vibration category.</t>
         </is>
       </c>
       <c r="AQ26" s="223" t="inlineStr">
@@ -3813,28 +3805,28 @@
       </c>
       <c r="AR26" s="223" t="inlineStr">
         <is>
-          <t>A = Use an EC-nutrunner with torque/angle/rundown monitoring and fastener count OK/NOK interlock that blocks station completion unless each headlamp screw reaches 6 Nm within angle window.
-If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
-B = Add an in-station machine-vision gap/flushness measurement with interlock that prevents proceeding unless gap/flushness at defined points is within specification.
-If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
+          <t>A = Add an in-station DC electric torque tool with OK/NOK (torque + angle) and screw-present sensing interlocked so the station cannot complete unless all headlamp screws reach 6 Nm within window.
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode in-station and prevent further processing)
+B = Install an in-station machine-vision gap/flush measurement with automatic NOK interlock that prevents completion/transfer if any measured gap is out of tolerance.
+If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing)</t>
         </is>
       </c>
       <c r="AS26" s="223" t="inlineStr">
         <is>
-          <t>A = Add a dedicated headlamp locating fixture with BIW datum hard-stops/dowel pins to set uniform fender gaps before fastening so the screw holes align and cross-threading/failed fit cannot occur.
-B = Introduce a simple 3-point gap/flushness locator fixture or go/no-go gap shims to hold the headlamp to the specified gaps against the fender/BIW while bolts are torqued to 6 Nm.</t>
+          <t>A = Install a simple alignment/locator fixture or pins that index the headlamp to BIW datums and hold uniform gaps before bolt insertion so screws start straight and can be properly torqued.
+B = Add a simple in-station gap/flushness setting aid (e.g., dedicated alignment locators plus go/no-go gap shims used during tightening) so the headlamp is constrained to the specified uniform gap before torque is applied.</t>
         </is>
       </c>
       <c r="AT26" s="223" t="inlineStr">
         <is>
           <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.
-- Cause/Mode mismatch: The stated Cause addresses only non-uniform gaps, not the 'failed to fit screws' portion of the Mode.</t>
+- Cause/Mode mismatch: The stated Cause addresses only gap non-uniformity and does not explain the 'failed to fit screws' part of the Mode.</t>
         </is>
       </c>
       <c r="AU26" s="223" t="inlineStr">
         <is>
-          <t>- Missing: Ship-to-Plant effect
-- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+          <t>- Missing: Ship-to-Plant effect; Vague: Current Detection Controls
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing beam-alignment, reduced road visibility, accident-risk effects — review/add to this row's Effect cell if applicable.</t>
         </is>
       </c>
       <c r="AV26" s="223" t="inlineStr"/>
@@ -3973,21 +3965,21 @@
       </c>
       <c r="AO28" s="223" t="inlineStr">
         <is>
-          <t>For an under-torqued headlamp mount, the DIRECT end-user outcome listed is rattling/vibration noise while driving, which maps to very objectionable NVH. No explicit safety or regulatory consequence is stated, and other listed effects require additional, unstated failure steps.</t>
+          <t>The most direct End User effect of an under‑torqued headlamp mounting is rattling/vibration noise while driving, which matches the table’s NVH category for very objectionable sound/vibration (S=4). Other listed outcomes (cracked lens, bulb burnout, water ingress, eye strain) require additional unstated failure steps and are therefore indirect for this mode/cause.</t>
         </is>
       </c>
       <c r="AQ28" s="223" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AR28" s="223" t="inlineStr">
         <is>
-          <t>Add in-station torque transducer monitoring with the nutrunner controller that records OK/NOK per bolt and stops the station or prevents advancement on any NOK torque.
-If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)</t>
+          <t>Add in‑station torque/angle monitoring with the tool controller providing OK/NOK and blocking job completion or advancing the line if target torque is not reached.
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing or automatically routes discrepant product to reject.)</t>
         </is>
       </c>
       <c r="AS28" s="223" t="inlineStr">
         <is>
-          <t>Install a controller-based DC nutrunner for the headlamp bolts with program-locked 6 Nm, socket/tool ID verification, bolt-count, and OK/NOK interlock to prevent job completion unless torque is achieved.</t>
+          <t>Install a controller‑managed DC nutrunner for this joint with auto program selection by part scan and lockout on wrong tool or out‑of‑calibration status to ensure 6 Nm is achieved.</t>
         </is>
       </c>
       <c r="AT28" s="223" t="inlineStr">
@@ -3998,12 +3990,12 @@
       <c r="AU28" s="223" t="inlineStr">
         <is>
           <t>- Missing: Ship-to-Plant effect
-- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment and reduced visibility/accident-risk effects — review/add to this row's Effect cell if applicable.</t>
         </is>
       </c>
       <c r="AV28" s="223" t="inlineStr"/>
     </row>
-    <row r="29" ht="240" customFormat="1" customHeight="1" s="13">
+    <row r="29" ht="285" customFormat="1" customHeight="1" s="13">
       <c r="B29" s="210" t="n"/>
       <c r="C29" s="211" t="n"/>
       <c r="D29" s="210" t="n"/>
@@ -4044,20 +4036,20 @@
       <c r="AL29" s="10" t="n"/>
       <c r="AM29" s="223" t="inlineStr">
         <is>
-          <t>A = Under-torque (torque not achieved)
-B = Over-torque</t>
+          <t>A = TORQUE NOT ACHIEVED
+B = OVER TORQUE</t>
         </is>
       </c>
       <c r="AN29" s="223" t="inlineStr">
         <is>
           <t>A = 4
-B = 7</t>
+B = 4</t>
         </is>
       </c>
       <c r="AO29" s="223" t="inlineStr">
         <is>
-          <t>A = For under-torque of the headlamp mounting, the only direct end-user effect listed is rattling/vibration during driving, which is an NVH complaint. Per the table, objectionable noise/vibration maps to Severity 4. Other listed effects (crack, burnout, water ingress, eye strain) require additional unstated failure steps and are indirect for this mode/cause.
-B = The direct end user effect of over‑torque is a cracked/broken lens, which would degrade headlamp performance rather than eliminate it entirely. No accident/injury or regulatory language is stated, so this aligns with degraded primary function.</t>
+          <t>A = The direct end user outcome of a headlamp mounting joint not achieving torque is rattling/vibration noise while driving, which fits the table’s NVH category. Other listed outcomes (bulb burnout, water ingress, lens crack) require additional unstated mechanisms beyond a torque miss and are therefore not representative for this mode/cause.
+B = Among the End User effects, the direct outcome of over-torque is a loose/damaged joint causing “rattling or vibration noise during driving,” which maps to very objectionable NVH. No safety or regulatory language is stated, and other listed effects require additional unstated failure steps.</t>
         </is>
       </c>
       <c r="AQ29" s="223" t="inlineStr">
@@ -4068,16 +4060,16 @@
       </c>
       <c r="AR29" s="223" t="inlineStr">
         <is>
-          <t>A = Install a controller-monitored DC nutrunner with torque/angle monitoring and OK/NOK interlock that prevents station completion if 6 Nm is not achieved.
-If adopted, Detection = 3 (Machine-based automated detection method that will detect the failure mode IN-STATION and prevent further processing (D3).)
-B = Add in‑station torque/angle monitoring with automatic NOK lockout that stops processing if any headlamp fastener exceeds the upper torque limit.
-If adopted, Detection = 2 (Machine-based detection method that will detect the CAUSE and PREVENT the failure mode (discrepant part) from being produced (D2).)</t>
+          <t>A = Add in-station transducerized torque monitoring with automatic OK/NOK interlock and data logging so any under-/over-torque is detected and the line is stopped before the vehicle leaves the station.
+If adopted, Detection = 3 (Machine-based automated detection in-station that prevents further processing/outflow)
+B = Add in-station torque monitoring with a transducer-based OK/NOK judgment that interlocks the station (rejects the part/stops processing) if final torque exceeds the upper limit.
+If adopted, Detection = 3 (Machine-based automated detection in-station that stops further processing and prevents outflow; proven/standard torque monitoring method.)</t>
         </is>
       </c>
       <c r="AS29" s="223" t="inlineStr">
         <is>
-          <t>A = Add a tool-ID and calibration-status interlock tied to part scan so only the correct, in-calibration 6 Nm DC nutrunner can run this operation and all other tools are locked out.
-B = Replace the labeled dedicated gun with a transducerized shut‑off torque tool programmed to 6 Nm with an upper torque limit and PLC interlock that blocks the cycle on NOK/tool‑mismatch and logs torque results.</t>
+          <t>A = Install a DC electric torque tool with integrated controller and socket/tool-ID lockout tied to the 6 Nm program so only the correct tool can run and the joint cannot be completed unless target torque is achieved.
+B = Install a controller-managed DC torque tool programmed to 6 Nm with an upper torque limit and line interlock/lockout so fastenings outside spec cannot be completed or are automatically blocked.</t>
         </is>
       </c>
       <c r="AT29" s="223" t="inlineStr">
@@ -4089,7 +4081,7 @@
       <c r="AU29" s="223" t="inlineStr">
         <is>
           <t>- Missing: Ship-to-Plant effect
-- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced visibility, accident-risk effects; review/add to this row's Effect cell if applicable.</t>
+- Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment and reduced visibility/accident-risk effects — review/add to this row's Effect cell if applicable.</t>
         </is>
       </c>
       <c r="AV29" s="223" t="inlineStr"/>

</xml_diff>